<commit_message>
ParameterRetriever: Implemented possibility to reference external csv-files with data in the parameter Excel-files
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FertiliserMgmt.xlsx
+++ b/data/prod_parameters/FertiliserMgmt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>f_crop</t>
   </si>
@@ -76,8 +76,17 @@
     </r>
   </si>
   <si>
+    <t>N_c</t>
+  </si>
+  <si>
+    <t>N_n</t>
+  </si>
+  <si>
+    <t>Höstvete bröd, södra götaland</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">N recommendation as a function of yield </t>
+      <t xml:space="preserve">N recommendation [kg-N / ha (??)] as a function of yield </t>
     </r>
     <r>
       <rPr>
@@ -89,12 +98,6 @@
       </rPr>
       <t>( N_rec = N_a*Y^2 + N_b*Y + N_m )</t>
     </r>
-  </si>
-  <si>
-    <t>N_c</t>
-  </si>
-  <si>
-    <t>N_n</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -494,6 +497,9 @@
       <c r="D3">
         <v>-0.71430000000000005</v>
       </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -533,15 +539,21 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>-0.32340000000000002</v>
       </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>0.97240000000000004</v>

</xml_diff>

<commit_message>
Work in progress on method to calculate N application
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FertiliserMgmt.xlsx
+++ b/data/prod_parameters/FertiliserMgmt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="27">
   <si>
     <t>f_crop</t>
   </si>
@@ -49,16 +49,31 @@
     <t>f_fert_region</t>
   </si>
   <si>
-    <t>N_a</t>
-  </si>
-  <si>
-    <t>N_b</t>
-  </si>
-  <si>
-    <t>N_m</t>
-  </si>
-  <si>
     <t>Wheat, winter</t>
+  </si>
+  <si>
+    <t>f_use</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>N_rec_a</t>
+  </si>
+  <si>
+    <t>N_rec_b</t>
+  </si>
+  <si>
+    <t>N_rec_m</t>
+  </si>
+  <si>
+    <t>N_ley_a</t>
+  </si>
+  <si>
+    <t>N_ley_m</t>
+  </si>
+  <si>
+    <t>Höstevete norra götaland och svealand</t>
   </si>
   <si>
     <r>
@@ -72,17 +87,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>( N_app = N_rec * (N_c*PL + N_n) )</t>
+      <t>( N_app = N_rec * (N_ley_a*PL + N_ley_m) )</t>
     </r>
-  </si>
-  <si>
-    <t>N_c</t>
-  </si>
-  <si>
-    <t>N_n</t>
-  </si>
-  <si>
-    <t>Höstvete bröd, södra götaland</t>
   </si>
   <si>
     <r>
@@ -96,15 +102,39 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>( N_rec = N_a*Y^2 + N_b*Y + N_m )</t>
+      <t>( N_rec = N_rec_a*Y^2 + N_rec_b*Y + N_rec_m )</t>
     </r>
+  </si>
+  <si>
+    <t>Fallback</t>
+  </si>
+  <si>
+    <t>Wheat, spring</t>
+  </si>
+  <si>
+    <t>Barley, spring</t>
+  </si>
+  <si>
+    <t>Korn, foder, norra götaland och svealand</t>
+  </si>
+  <si>
+    <t>Korn, malt norra götaland och svealand</t>
+  </si>
+  <si>
+    <t>Havre, norra götaland och svealand</t>
+  </si>
+  <si>
+    <t>Oats</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0E+00"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +155,26 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -156,11 +206,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,123 +494,407 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" customWidth="1"/>
-    <col min="6" max="6" width="35.42578125" customWidth="1"/>
-    <col min="7" max="7" width="27.42578125" customWidth="1"/>
+    <col min="1" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" customWidth="1"/>
+    <col min="7" max="7" width="35.42578125" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="F2" s="2"/>
       <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" s="5">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
-        <v>-0.71430000000000005</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>-0.80359999999999998</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>24.088999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8">
+        <v>55.213999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9">
+        <v>50.213999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12">
+        <v>-1.0713999999999999</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13">
+        <v>23.928999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="6">
+        <v>1E-13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18">
+        <v>-1.0713999999999999</v>
+      </c>
+      <c r="G18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19">
+        <v>23.928999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D24" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D25" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>23.143000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>47.570999999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8">
+      <c r="E25" s="5">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26">
         <v>-0.32340000000000002</v>
       </c>
-      <c r="F8" t="s">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="E27">
+        <v>0.97240000000000004</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" t="s">
         <v>15</v>
       </c>
-      <c r="D9">
-        <v>0.97240000000000004</v>
-      </c>
+      <c r="E28">
+        <v>-0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29">
+        <v>0.81369999999999998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30">
+        <v>-0.41710000000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D31" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31">
+        <v>0.91610000000000003</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32">
+        <v>-0.74150000000000005</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33">
+        <v>0.96550000000000002</v>
+      </c>
+    </row>
+    <row r="55" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K55" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed bug in N req calc. and updated equation parameters
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FertiliserMgmt.xlsx
+++ b/data/prod_parameters/FertiliserMgmt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="relations" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="112">
   <si>
     <t>f_crop</t>
   </si>
@@ -262,9 +262,6 @@
     <t>Assume 94% of recommended N, based on average in Sweden. Very little statistics available</t>
   </si>
   <si>
-    <t>inte minus i Hannas dokument??</t>
-  </si>
-  <si>
     <t>recommended nitrogen rate is 110 kg N/ha, which is followed more or less according to statistics (applied N rates (plant available N) were 98-105% of recommended rate in 2016)</t>
   </si>
   <si>
@@ -293,12 +290,6 @@
   </si>
   <si>
     <t xml:space="preserve">yield in fresh weight 5% DM </t>
-  </si>
-  <si>
-    <t>same as table potatoes?</t>
-  </si>
-  <si>
-    <t>Avser "Majs" i dokumentet grönfoder eller tröskad?</t>
   </si>
   <si>
     <t>f_prod_system</t>
@@ -383,6 +374,12 @@
   </si>
   <si>
     <t>Havre södra götaland</t>
+  </si>
+  <si>
+    <t>Korn, norrland</t>
+  </si>
+  <si>
+    <t>Potatis</t>
   </si>
 </sst>
 </file>
@@ -771,13 +768,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L211"/>
+  <dimension ref="A1:L224"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="7.28515625" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.42578125" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="8.140625" customWidth="1"/>
@@ -793,10 +790,10 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -816,7 +813,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -874,7 +871,7 @@
         <v>-0.80359999999999998</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -918,7 +915,7 @@
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -927,7 +924,7 @@
         <v>-0.71430000000000005</v>
       </c>
       <c r="H10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -935,7 +932,7 @@
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
@@ -949,7 +946,7 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E12" t="s">
         <v>12</v>
@@ -966,7 +963,7 @@
         <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
@@ -980,7 +977,7 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -999,7 +996,7 @@
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
@@ -1014,7 +1011,7 @@
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E16" t="s">
         <v>12</v>
@@ -1032,7 +1029,7 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E17" t="s">
         <v>12</v>
@@ -1105,7 +1102,7 @@
         <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1114,7 +1111,7 @@
         <v>-1.25</v>
       </c>
       <c r="H23" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1122,7 +1119,7 @@
         <v>27</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E24" t="s">
         <v>11</v>
@@ -1136,7 +1133,7 @@
         <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E25" t="s">
         <v>12</v>
@@ -1150,7 +1147,7 @@
         <v>27</v>
       </c>
       <c r="D26" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1170,7 +1167,7 @@
         <v>27</v>
       </c>
       <c r="D27" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E27" t="s">
         <v>11</v>
@@ -1187,7 +1184,7 @@
         <v>27</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E28" t="s">
         <v>12</v>
@@ -1229,7 +1226,7 @@
         <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1238,7 +1235,7 @@
         <v>-0.71430000000000005</v>
       </c>
       <c r="H31" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1246,7 +1243,7 @@
         <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
         <v>11</v>
@@ -1260,7 +1257,7 @@
         <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E33" t="s">
         <v>12</v>
@@ -1274,7 +1271,7 @@
         <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1293,7 +1290,7 @@
         <v>23</v>
       </c>
       <c r="D35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
@@ -1308,7 +1305,7 @@
         <v>23</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E36" t="s">
         <v>12</v>
@@ -1404,7 +1401,7 @@
         <v>17</v>
       </c>
       <c r="D43" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E43" t="s">
         <v>10</v>
@@ -1413,7 +1410,7 @@
         <v>-1.25</v>
       </c>
       <c r="H43" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -1421,7 +1418,7 @@
         <v>17</v>
       </c>
       <c r="D44" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E44" t="s">
         <v>11</v>
@@ -1435,7 +1432,7 @@
         <v>17</v>
       </c>
       <c r="D45" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E45" t="s">
         <v>12</v>
@@ -1452,7 +1449,7 @@
         <v>9</v>
       </c>
       <c r="D46" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E46" t="s">
         <v>10</v>
@@ -1461,7 +1458,7 @@
         <v>-2E-12</v>
       </c>
       <c r="H46" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -1472,7 +1469,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E47" t="s">
         <v>11</v>
@@ -1489,7 +1486,7 @@
         <v>9</v>
       </c>
       <c r="D48" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E48" t="s">
         <v>12</v>
@@ -1503,13 +1500,13 @@
         <v>17</v>
       </c>
       <c r="D49" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E49" t="s">
         <v>10</v>
       </c>
       <c r="F49" s="9">
-        <f>F43</f>
+        <f t="shared" ref="F49:F54" si="1">F43</f>
         <v>-1.25</v>
       </c>
       <c r="H49" s="9" t="str">
@@ -1522,13 +1519,13 @@
         <v>17</v>
       </c>
       <c r="D50" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E50" t="s">
         <v>11</v>
       </c>
       <c r="F50" s="9">
-        <f>F44</f>
+        <f t="shared" si="1"/>
         <v>25.25</v>
       </c>
     </row>
@@ -1537,13 +1534,13 @@
         <v>17</v>
       </c>
       <c r="D51" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E51" t="s">
         <v>12</v>
       </c>
       <c r="F51" s="9">
-        <f>F45</f>
+        <f t="shared" si="1"/>
         <v>19.75</v>
       </c>
     </row>
@@ -1555,13 +1552,13 @@
         <v>9</v>
       </c>
       <c r="D52" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E52" t="s">
         <v>10</v>
       </c>
       <c r="F52" s="9">
-        <f>F46</f>
+        <f t="shared" si="1"/>
         <v>-2E-12</v>
       </c>
       <c r="H52" s="9" t="str">
@@ -1577,13 +1574,13 @@
         <v>9</v>
       </c>
       <c r="D53" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E53" t="s">
         <v>11</v>
       </c>
       <c r="F53" s="9">
-        <f>F47</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
@@ -1595,100 +1592,122 @@
         <v>9</v>
       </c>
       <c r="D54" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E54" t="s">
         <v>12</v>
       </c>
       <c r="F54" s="9">
-        <f>F48</f>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="D55" t="s">
+        <v>99</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
       </c>
-      <c r="F55">
-        <v>-1.0713999999999999</v>
+      <c r="F55" s="5">
+        <v>0</v>
       </c>
       <c r="H55" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="D56" t="s">
+        <v>99</v>
       </c>
       <c r="E56" t="s">
         <v>11</v>
       </c>
-      <c r="F56">
-        <v>23.928999999999998</v>
+      <c r="F56" s="5">
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="D57" t="s">
+        <v>99</v>
       </c>
       <c r="E57" t="s">
         <v>12</v>
       </c>
-      <c r="F57">
-        <v>22</v>
+      <c r="F57" s="5">
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="B58" t="s">
+        <v>9</v>
       </c>
       <c r="D58" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
-      <c r="F58">
-        <v>-1.25</v>
-      </c>
-      <c r="H58" t="s">
-        <v>112</v>
+      <c r="F58" s="9">
+        <f t="shared" ref="F58:F66" si="2">F55</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="9" t="str">
+        <f>H55</f>
+        <v>Korn, norrland</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="B59" t="s">
+        <v>9</v>
       </c>
       <c r="D59" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E59" t="s">
         <v>11</v>
       </c>
-      <c r="F59">
-        <v>25.25</v>
+      <c r="F59" s="9">
+        <f t="shared" si="2"/>
+        <v>20</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="B60" t="s">
+        <v>9</v>
       </c>
       <c r="D60" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E60" t="s">
         <v>12</v>
       </c>
-      <c r="F60">
-        <v>9.75</v>
+      <c r="F60" s="9">
+        <f t="shared" si="2"/>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D61" t="s">
         <v>100</v>
@@ -1697,17 +1716,17 @@
         <v>10</v>
       </c>
       <c r="F61" s="9">
-        <f>F58</f>
-        <v>-1.25</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="H61" s="9" t="str">
         <f>H58</f>
-        <v>Havre södra götaland</v>
+        <v>Korn, norrland</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D62" t="s">
         <v>100</v>
@@ -1716,13 +1735,13 @@
         <v>11</v>
       </c>
       <c r="F62" s="9">
-        <f>F59</f>
-        <v>25.25</v>
+        <f t="shared" si="2"/>
+        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D63" t="s">
         <v>100</v>
@@ -1731,1373 +1750,1430 @@
         <v>12</v>
       </c>
       <c r="F63" s="9">
-        <f>F60</f>
-        <v>9.75</v>
+        <f t="shared" si="2"/>
+        <v>35</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>17</v>
+      </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" t="s">
+        <v>100</v>
+      </c>
+      <c r="E64" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H64" s="9" t="str">
+        <f>H61</f>
+        <v>Korn, norrland</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>17</v>
+      </c>
+      <c r="B65" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" t="s">
+        <v>100</v>
+      </c>
+      <c r="E65" t="s">
+        <v>11</v>
+      </c>
+      <c r="F65" s="9">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>17</v>
+      </c>
+      <c r="B66" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" t="s">
+        <v>100</v>
+      </c>
+      <c r="E66" t="s">
+        <v>12</v>
+      </c>
+      <c r="F66" s="9">
+        <f t="shared" si="2"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>21</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67">
+        <v>-1.0713999999999999</v>
+      </c>
+      <c r="H67" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>21</v>
+      </c>
+      <c r="E68" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68">
+        <v>23.928999999999998</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>21</v>
+      </c>
+      <c r="E69" t="s">
+        <v>12</v>
+      </c>
+      <c r="F69">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" t="s">
+        <v>98</v>
+      </c>
+      <c r="E70" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70">
+        <v>-1.25</v>
+      </c>
+      <c r="H70" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" t="s">
+        <v>98</v>
+      </c>
+      <c r="E71" t="s">
+        <v>11</v>
+      </c>
+      <c r="F71">
+        <v>25.25</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>21</v>
+      </c>
+      <c r="D72" t="s">
+        <v>98</v>
+      </c>
+      <c r="E72" t="s">
+        <v>12</v>
+      </c>
+      <c r="F72">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>21</v>
+      </c>
+      <c r="D73" t="s">
+        <v>97</v>
+      </c>
+      <c r="E73" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" s="9">
+        <f>F70</f>
+        <v>-1.25</v>
+      </c>
+      <c r="H73" s="9" t="str">
+        <f>H70</f>
+        <v>Havre södra götaland</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" t="s">
+        <v>97</v>
+      </c>
+      <c r="E74" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" s="9">
+        <f>F71</f>
+        <v>25.25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>21</v>
+      </c>
+      <c r="D75" t="s">
+        <v>97</v>
+      </c>
+      <c r="E75" t="s">
+        <v>12</v>
+      </c>
+      <c r="F75" s="9">
+        <f>F72</f>
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>25</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E76" t="s">
         <v>11</v>
       </c>
-      <c r="F64" s="9">
+      <c r="F76" s="9">
         <f>F29</f>
         <v>16.856999999999999</v>
       </c>
-      <c r="H64" s="9" t="str">
+      <c r="H76" s="9" t="str">
         <f>H29</f>
         <v>Rågvete/höstkorn, norra  götaland och svealand</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>25</v>
       </c>
-      <c r="E65" t="s">
-        <v>12</v>
-      </c>
-      <c r="F65" s="9">
+      <c r="E77" t="s">
+        <v>12</v>
+      </c>
+      <c r="F77" s="9">
         <f>F30</f>
         <v>59.143000000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>25</v>
       </c>
-      <c r="D66" t="s">
-        <v>101</v>
-      </c>
-      <c r="E66" t="s">
+      <c r="D78" t="s">
+        <v>98</v>
+      </c>
+      <c r="E78" t="s">
         <v>10</v>
       </c>
-      <c r="F66" s="9">
+      <c r="F78" s="9">
         <f>F34</f>
         <v>-0.71430000000000005</v>
       </c>
-      <c r="H66" s="9" t="str">
+      <c r="H78" s="9" t="str">
         <f>H34</f>
         <v>Rågvete/höstkorn, södra götaland</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>25</v>
       </c>
-      <c r="D67" t="s">
-        <v>101</v>
-      </c>
-      <c r="E67" t="s">
+      <c r="D79" t="s">
+        <v>98</v>
+      </c>
+      <c r="E79" t="s">
         <v>11</v>
       </c>
-      <c r="F67" s="9">
+      <c r="F79" s="9">
         <f>F35</f>
         <v>23.143000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>25</v>
       </c>
-      <c r="D68" t="s">
-        <v>101</v>
-      </c>
-      <c r="E68" t="s">
-        <v>12</v>
-      </c>
-      <c r="F68" s="9">
+      <c r="D80" t="s">
+        <v>98</v>
+      </c>
+      <c r="E80" t="s">
+        <v>12</v>
+      </c>
+      <c r="F80" s="9">
         <f>F36</f>
         <v>37.570999999999998</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>25</v>
       </c>
-      <c r="D69" t="s">
-        <v>100</v>
-      </c>
-      <c r="E69" t="s">
+      <c r="D81" t="s">
+        <v>97</v>
+      </c>
+      <c r="E81" t="s">
         <v>10</v>
       </c>
-      <c r="F69" s="9">
+      <c r="F81" s="9">
         <f>F34</f>
         <v>-0.71430000000000005</v>
       </c>
-      <c r="H69" s="9" t="str">
+      <c r="H81" s="9" t="str">
         <f>H34</f>
         <v>Rågvete/höstkorn, södra götaland</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>25</v>
       </c>
-      <c r="D70" t="s">
-        <v>100</v>
-      </c>
-      <c r="E70" t="s">
+      <c r="D82" t="s">
+        <v>97</v>
+      </c>
+      <c r="E82" t="s">
         <v>11</v>
       </c>
-      <c r="F70" s="9">
+      <c r="F82" s="9">
         <f>F35</f>
         <v>23.143000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>25</v>
       </c>
-      <c r="D71" t="s">
-        <v>100</v>
-      </c>
-      <c r="E71" t="s">
-        <v>12</v>
-      </c>
-      <c r="F71" s="9">
+      <c r="D83" t="s">
+        <v>97</v>
+      </c>
+      <c r="E83" t="s">
+        <v>12</v>
+      </c>
+      <c r="F83" s="9">
         <f>F36</f>
         <v>37.570999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>24</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E84" t="s">
         <v>11</v>
       </c>
-      <c r="F72" s="9">
+      <c r="F84" s="9">
         <f>F29</f>
         <v>16.856999999999999</v>
       </c>
-      <c r="H72" s="9" t="str">
+      <c r="H84" s="9" t="str">
         <f>H29</f>
         <v>Rågvete/höstkorn, norra  götaland och svealand</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>24</v>
       </c>
-      <c r="E73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F73" s="9">
+      <c r="E85" t="s">
+        <v>12</v>
+      </c>
+      <c r="F85" s="9">
         <f>F30</f>
         <v>59.143000000000001</v>
       </c>
-      <c r="H73" s="9"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+      <c r="H85" s="9"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>24</v>
       </c>
-      <c r="D74" t="s">
-        <v>101</v>
-      </c>
-      <c r="E74" t="s">
+      <c r="D86" t="s">
+        <v>98</v>
+      </c>
+      <c r="E86" t="s">
         <v>10</v>
       </c>
-      <c r="F74" s="9">
+      <c r="F86" s="9">
         <f>F34</f>
         <v>-0.71430000000000005</v>
       </c>
-      <c r="H74" s="9" t="str">
+      <c r="H86" s="9" t="str">
         <f>H34</f>
         <v>Rågvete/höstkorn, södra götaland</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>24</v>
       </c>
-      <c r="D75" t="s">
-        <v>101</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="D87" t="s">
+        <v>98</v>
+      </c>
+      <c r="E87" t="s">
         <v>11</v>
       </c>
-      <c r="F75" s="9">
+      <c r="F87" s="9">
         <f>F35</f>
         <v>23.143000000000001</v>
       </c>
-      <c r="H75" s="9"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="H87" s="9"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>24</v>
       </c>
-      <c r="D76" t="s">
-        <v>101</v>
-      </c>
-      <c r="E76" t="s">
-        <v>12</v>
-      </c>
-      <c r="F76" s="9">
+      <c r="D88" t="s">
+        <v>98</v>
+      </c>
+      <c r="E88" t="s">
+        <v>12</v>
+      </c>
+      <c r="F88" s="9">
         <f>F36</f>
         <v>37.570999999999998</v>
       </c>
-      <c r="H76" s="9"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="H88" s="9"/>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>24</v>
       </c>
-      <c r="D77" t="s">
-        <v>100</v>
-      </c>
-      <c r="E77" t="s">
+      <c r="D89" t="s">
+        <v>97</v>
+      </c>
+      <c r="E89" t="s">
         <v>10</v>
       </c>
-      <c r="F77" s="9">
+      <c r="F89" s="9">
         <f>F34</f>
         <v>-0.71430000000000005</v>
       </c>
-      <c r="H77" s="9" t="str">
+      <c r="H89" s="9" t="str">
         <f>H34</f>
         <v>Rågvete/höstkorn, södra götaland</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>24</v>
       </c>
-      <c r="D78" t="s">
-        <v>100</v>
-      </c>
-      <c r="E78" t="s">
+      <c r="D90" t="s">
+        <v>97</v>
+      </c>
+      <c r="E90" t="s">
         <v>11</v>
       </c>
-      <c r="F78" s="9">
+      <c r="F90" s="9">
         <f>F35</f>
         <v>23.143000000000001</v>
       </c>
-      <c r="H78" s="9"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+      <c r="H90" s="9"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>24</v>
       </c>
-      <c r="D79" t="s">
-        <v>100</v>
-      </c>
-      <c r="E79" t="s">
-        <v>12</v>
-      </c>
-      <c r="F79" s="9">
+      <c r="D91" t="s">
+        <v>97</v>
+      </c>
+      <c r="E91" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="9">
         <f>F36</f>
         <v>37.570999999999998</v>
       </c>
-      <c r="H79" s="9"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A80" s="7" t="s">
+      <c r="H91" s="9"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E80" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F80" s="7">
-        <v>-1.7857000000000001</v>
-      </c>
-      <c r="H80" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A81" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E81" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F81" s="7">
-        <v>43.570999999999998</v>
-      </c>
-      <c r="H81" s="7"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A82" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F82" s="7">
-        <v>-112.5</v>
-      </c>
-      <c r="H82" s="7"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>28</v>
-      </c>
-      <c r="E83" t="s">
-        <v>12</v>
-      </c>
-      <c r="F83">
-        <v>50</v>
-      </c>
-      <c r="H83" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>30</v>
-      </c>
-      <c r="E84" t="s">
-        <v>12</v>
-      </c>
-      <c r="F84">
-        <v>0</v>
-      </c>
-      <c r="H84" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>31</v>
-      </c>
-      <c r="E85" t="s">
-        <v>12</v>
-      </c>
-      <c r="F85">
-        <v>0</v>
-      </c>
-      <c r="H85" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>32</v>
-      </c>
-      <c r="E86" t="s">
-        <v>12</v>
-      </c>
-      <c r="F86">
-        <v>0</v>
-      </c>
-      <c r="H86" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>33</v>
-      </c>
-      <c r="E87" t="s">
-        <v>12</v>
-      </c>
-      <c r="F87">
-        <v>30</v>
-      </c>
-      <c r="H87" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>34</v>
-      </c>
-      <c r="E88" t="s">
-        <v>11</v>
-      </c>
-      <c r="F88">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>34</v>
-      </c>
-      <c r="E89" t="s">
-        <v>12</v>
-      </c>
-      <c r="F89">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>35</v>
-      </c>
-      <c r="E90" t="s">
-        <v>11</v>
-      </c>
-      <c r="F90">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>35</v>
-      </c>
-      <c r="E91" t="s">
-        <v>12</v>
-      </c>
-      <c r="F91">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>36</v>
-      </c>
-      <c r="E92" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92">
-        <v>-2.5000000000000001E-2</v>
-      </c>
+      <c r="E92" s="7"/>
+      <c r="F92" s="7"/>
+      <c r="H92" s="7"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E93" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F93">
-        <v>4.95</v>
+        <v>50</v>
+      </c>
+      <c r="H93" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E94" t="s">
         <v>12</v>
       </c>
       <c r="F94">
-        <v>-31.5</v>
+        <v>0</v>
+      </c>
+      <c r="H94" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E95" t="s">
-        <v>10</v>
-      </c>
-      <c r="F95" s="9">
-        <f>F92</f>
-        <v>-2.5000000000000001E-2</v>
-      </c>
-      <c r="H95" s="7" t="s">
-        <v>91</v>
+        <v>12</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="H95" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>32</v>
+      </c>
+      <c r="E96" t="s">
+        <v>12</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="H96" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>33</v>
+      </c>
+      <c r="E97" t="s">
+        <v>12</v>
+      </c>
+      <c r="F97">
+        <v>30</v>
+      </c>
+      <c r="H97" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>34</v>
+      </c>
+      <c r="E98" t="s">
+        <v>11</v>
+      </c>
+      <c r="F98">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>34</v>
+      </c>
+      <c r="E99" t="s">
+        <v>12</v>
+      </c>
+      <c r="F99">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>35</v>
+      </c>
+      <c r="E100" t="s">
+        <v>11</v>
+      </c>
+      <c r="F100">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>35</v>
+      </c>
+      <c r="E101" t="s">
+        <v>12</v>
+      </c>
+      <c r="F101">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>36</v>
+      </c>
+      <c r="E102" t="s">
+        <v>10</v>
+      </c>
+      <c r="F102">
+        <v>-2.5000000000000001E-2</v>
+      </c>
+      <c r="H102" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>36</v>
+      </c>
+      <c r="E103" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103">
+        <v>4.95</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>36</v>
+      </c>
+      <c r="E104" t="s">
+        <v>12</v>
+      </c>
+      <c r="F104">
+        <v>-31.5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>37</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E105" t="s">
+        <v>10</v>
+      </c>
+      <c r="F105" s="9">
+        <f>F102</f>
+        <v>-2.5000000000000001E-2</v>
+      </c>
+      <c r="H105" s="9" t="str">
+        <f>H102</f>
+        <v>Potatis</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>37</v>
+      </c>
+      <c r="E106" t="s">
         <v>11</v>
       </c>
-      <c r="F96" s="9">
-        <f t="shared" ref="F96:F97" si="1">F93</f>
+      <c r="F106" s="9">
+        <f t="shared" ref="F106:F107" si="3">F103</f>
         <v>4.95</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>37</v>
       </c>
-      <c r="E97" t="s">
-        <v>12</v>
-      </c>
-      <c r="F97" s="9">
-        <f t="shared" si="1"/>
+      <c r="E107" t="s">
+        <v>12</v>
+      </c>
+      <c r="F107" s="9">
+        <f t="shared" si="3"/>
         <v>-31.5</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>38</v>
       </c>
-      <c r="E98" t="s">
-        <v>12</v>
-      </c>
-      <c r="F98">
+      <c r="E108" t="s">
+        <v>12</v>
+      </c>
+      <c r="F108">
         <v>110</v>
       </c>
-      <c r="H98" t="s">
+      <c r="H108" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E110" t="s">
+        <v>10</v>
+      </c>
+      <c r="F110">
+        <v>-1.4286000000000001</v>
+      </c>
+      <c r="H110" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="10" t="s">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E100" t="s">
-        <v>10</v>
-      </c>
-      <c r="F100">
-        <v>-1.4286000000000001</v>
-      </c>
-      <c r="H100" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" s="10" t="s">
+      <c r="E111" t="s">
+        <v>11</v>
+      </c>
+      <c r="F111">
+        <v>40.713999999999999</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E101" t="s">
-        <v>11</v>
-      </c>
-      <c r="F101">
-        <v>40.713999999999999</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E102" t="s">
-        <v>12</v>
-      </c>
-      <c r="F102">
+      <c r="E112" t="s">
+        <v>12</v>
+      </c>
+      <c r="F112">
         <v>-74.856999999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" s="11" t="s">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A104" s="5" t="s">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E104" t="s">
-        <v>12</v>
-      </c>
-      <c r="F104">
+      <c r="E114" t="s">
+        <v>12</v>
+      </c>
+      <c r="F114">
         <v>0</v>
       </c>
-      <c r="H104" t="s">
+      <c r="H114" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A105" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E105" s="7"/>
-      <c r="F105" s="7"/>
-      <c r="H105" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" s="11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A107" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A108" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="E108" t="s">
-        <v>12</v>
-      </c>
-      <c r="F108">
-        <v>0</v>
-      </c>
-      <c r="H108" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E109" t="s">
-        <v>12</v>
-      </c>
-      <c r="F109">
-        <v>0</v>
-      </c>
-      <c r="H109" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>47</v>
-      </c>
-      <c r="E110" t="s">
-        <v>11</v>
-      </c>
-      <c r="F110">
-        <v>2.5</v>
-      </c>
-      <c r="H110" t="s">
-        <v>86</v>
-      </c>
-      <c r="I110" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>47</v>
-      </c>
-      <c r="E111" t="s">
-        <v>12</v>
-      </c>
-      <c r="F111">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>48</v>
-      </c>
-      <c r="E112" t="s">
-        <v>11</v>
-      </c>
-      <c r="F112">
-        <v>1.3846000000000001</v>
-      </c>
-      <c r="H112" t="s">
-        <v>86</v>
-      </c>
-      <c r="I112" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>48</v>
-      </c>
-      <c r="E113" t="s">
-        <v>12</v>
-      </c>
-      <c r="F113">
-        <v>11.538</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="7" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E115" t="s">
-        <v>11</v>
-      </c>
-      <c r="F115">
-        <v>3.3332999999999999</v>
-      </c>
-      <c r="H115" t="s">
-        <v>88</v>
-      </c>
-      <c r="I115" t="s">
-        <v>87</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B115" s="5"/>
+      <c r="C115" s="5"/>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F115" s="5">
+        <v>-1.7857000000000001</v>
+      </c>
+      <c r="H115" s="7"/>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E116" t="s">
-        <v>12</v>
-      </c>
-      <c r="F116">
-        <v>33.332999999999998</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B116" s="5"/>
+      <c r="C116" s="5"/>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" s="5">
+        <v>43.570999999999998</v>
+      </c>
+      <c r="H116" s="7"/>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E117" t="s">
+        <v>42</v>
+      </c>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F117" s="5">
+        <v>-112.5</v>
+      </c>
+      <c r="H117" s="7"/>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A118" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E120" t="s">
+        <v>12</v>
+      </c>
+      <c r="F120">
+        <v>0</v>
+      </c>
+      <c r="H120" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A121" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E121" t="s">
+        <v>12</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+      <c r="H121" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>47</v>
+      </c>
+      <c r="E122" t="s">
         <v>11</v>
       </c>
-      <c r="F117">
-        <v>3</v>
-      </c>
-      <c r="H117" t="s">
-        <v>89</v>
-      </c>
-      <c r="I117" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E118" t="s">
-        <v>12</v>
-      </c>
-      <c r="F118">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A119" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E119" t="s">
+      <c r="F122">
+        <v>2.5</v>
+      </c>
+      <c r="H122" t="s">
+        <v>85</v>
+      </c>
+      <c r="I122" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>47</v>
+      </c>
+      <c r="E123" t="s">
+        <v>12</v>
+      </c>
+      <c r="F123">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>48</v>
+      </c>
+      <c r="E124" t="s">
         <v>11</v>
       </c>
-      <c r="F119">
-        <v>2.6667000000000001</v>
-      </c>
-      <c r="H119" t="s">
-        <v>90</v>
-      </c>
-      <c r="I119" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A120" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E120" t="s">
-        <v>12</v>
-      </c>
-      <c r="F120">
-        <v>-43.332999999999998</v>
-      </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A121" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E121" t="s">
-        <v>11</v>
-      </c>
-      <c r="F121" s="9">
-        <f>F119</f>
-        <v>2.6667000000000001</v>
-      </c>
-      <c r="G121" s="9"/>
-      <c r="H121" s="9" t="str">
-        <f>H119</f>
-        <v xml:space="preserve">yield in fresh weight 5% DM </v>
-      </c>
-      <c r="I121" s="9" t="str">
-        <f>I119</f>
-        <v>Yara (2018)</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E122" t="s">
-        <v>12</v>
-      </c>
-      <c r="F122" s="9">
-        <f>F120</f>
-        <v>-43.332999999999998</v>
-      </c>
-      <c r="G122" s="9"/>
-      <c r="H122" s="9"/>
-      <c r="I122" s="9"/>
-    </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A123" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A124" s="7" t="s">
-        <v>55</v>
+      <c r="F124">
+        <v>1.3846000000000001</v>
+      </c>
+      <c r="H124" t="s">
+        <v>85</v>
+      </c>
+      <c r="I124" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="5" t="s">
-        <v>56</v>
+      <c r="A125" t="s">
+        <v>48</v>
       </c>
       <c r="E125" t="s">
         <v>12</v>
       </c>
       <c r="F125">
-        <v>65</v>
-      </c>
-      <c r="H125" t="s">
-        <v>83</v>
+        <v>11.538</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E127" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F127">
-        <v>65</v>
+        <v>3.3332999999999999</v>
       </c>
       <c r="H127" t="s">
-        <v>84</v>
+        <v>87</v>
+      </c>
+      <c r="I127" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E128" t="s">
         <v>12</v>
       </c>
       <c r="F128">
-        <v>100</v>
-      </c>
-      <c r="H128" t="s">
-        <v>85</v>
+        <v>33.332999999999998</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E129" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F129">
-        <v>110</v>
+        <v>3</v>
+      </c>
+      <c r="H129" t="s">
+        <v>88</v>
+      </c>
+      <c r="I129" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A130" s="7" t="s">
-        <v>61</v>
+      <c r="A130" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E130" t="s">
+        <v>12</v>
+      </c>
+      <c r="F130">
+        <v>90</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" s="7" t="s">
-        <v>62</v>
+      <c r="A131" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F131">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H131" t="s">
+        <v>89</v>
+      </c>
+      <c r="I131" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A132" s="7" t="s">
-        <v>63</v>
+      <c r="A132" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E132" t="s">
+        <v>11</v>
+      </c>
+      <c r="F132">
+        <v>1.2583</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A133" s="7" t="s">
-        <v>64</v>
+      <c r="A133" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E133" t="s">
+        <v>12</v>
+      </c>
+      <c r="F133">
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A134" s="7" t="s">
-        <v>65</v>
+      <c r="A134" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F134" s="9">
+        <f>F131</f>
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H134" s="9" t="str">
+        <f>H131</f>
+        <v xml:space="preserve">yield in fresh weight 5% DM </v>
+      </c>
+      <c r="I134" s="9" t="str">
+        <f>I131</f>
+        <v>Yara (2018)</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A135" s="7" t="s">
-        <v>66</v>
-      </c>
+      <c r="A135" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E135" t="s">
+        <v>11</v>
+      </c>
+      <c r="F135" s="9">
+        <f>F132</f>
+        <v>1.2583</v>
+      </c>
+      <c r="G135" s="9"/>
+      <c r="H135" s="9"/>
+      <c r="I135" s="9"/>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A136" s="7" t="s">
-        <v>67</v>
-      </c>
+      <c r="A136" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E136" t="s">
+        <v>12</v>
+      </c>
+      <c r="F136" s="9">
+        <f>F133</f>
+        <v>0</v>
+      </c>
+      <c r="G136" s="9"/>
+      <c r="H136" s="9"/>
+      <c r="I136" s="9"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E138" t="s">
-        <v>12</v>
-      </c>
-      <c r="F138">
-        <v>0</v>
-      </c>
-      <c r="H138" t="s">
-        <v>74</v>
+      <c r="A138" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A139" s="7" t="s">
-        <v>70</v>
+      <c r="A139" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E139" t="s">
+        <v>12</v>
+      </c>
+      <c r="F139">
+        <v>65</v>
+      </c>
+      <c r="H139" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E141" t="s">
+        <v>12</v>
+      </c>
+      <c r="F141">
+        <v>65</v>
+      </c>
+      <c r="H141" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E142" t="s">
+        <v>12</v>
+      </c>
+      <c r="F142">
+        <v>100</v>
+      </c>
+      <c r="H142" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E143" t="s">
+        <v>12</v>
+      </c>
+      <c r="F143">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A145" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A146" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A147" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A148" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A149" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A150" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A151" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A152" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E152" t="s">
+        <v>12</v>
+      </c>
+      <c r="F152">
+        <v>0</v>
+      </c>
+      <c r="H152" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A153" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A154" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A155" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E141" t="s">
-        <v>12</v>
-      </c>
-      <c r="F141">
+      <c r="E155" t="s">
+        <v>12</v>
+      </c>
+      <c r="F155">
         <v>0</v>
       </c>
-      <c r="H141" t="s">
+      <c r="H155" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B143" s="2"/>
-      <c r="C143" s="2"/>
-      <c r="D143" s="2"/>
-      <c r="E143" s="2"/>
-      <c r="F143" s="2"/>
-      <c r="G143" s="2"/>
-      <c r="H143" s="3"/>
-      <c r="I143" s="3"/>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E144" s="6" t="s">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B157" s="2"/>
+      <c r="C157" s="2"/>
+      <c r="D157" s="2"/>
+      <c r="E157" s="2"/>
+      <c r="F157" s="2"/>
+      <c r="G157" s="2"/>
+      <c r="H157" s="3"/>
+      <c r="I157" s="3"/>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E158" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F144" s="6">
+      <c r="F158" s="6">
         <v>0</v>
       </c>
-      <c r="G144" s="6"/>
-      <c r="H144" s="6" t="s">
+      <c r="G158" s="6"/>
+      <c r="H158" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E145" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F145" s="6">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E159" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F159" s="6">
         <v>1</v>
       </c>
-      <c r="G145" s="6"/>
-      <c r="H145" s="6" t="s">
+      <c r="G159" s="6"/>
+      <c r="H159" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>7</v>
-      </c>
-      <c r="E146" t="s">
-        <v>13</v>
-      </c>
-      <c r="F146">
-        <v>-0.32340000000000002</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>7</v>
-      </c>
-      <c r="E147" t="s">
-        <v>14</v>
-      </c>
-      <c r="F147">
-        <v>0.97240000000000004</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>16</v>
-      </c>
-      <c r="E148" t="s">
-        <v>13</v>
-      </c>
-      <c r="F148">
-        <v>-0.32500000000000001</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>16</v>
-      </c>
-      <c r="E149" t="s">
-        <v>14</v>
-      </c>
-      <c r="F149">
-        <v>0.81369999999999998</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>27</v>
-      </c>
-      <c r="E150" t="s">
-        <v>13</v>
-      </c>
-      <c r="F150">
-        <v>-0.58699999999999997</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>27</v>
-      </c>
-      <c r="E151" t="s">
-        <v>14</v>
-      </c>
-      <c r="F151">
-        <v>0.82350000000000001</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>23</v>
-      </c>
-      <c r="E152" t="s">
-        <v>13</v>
-      </c>
-      <c r="F152">
-        <v>-0.35070000000000001</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>23</v>
-      </c>
-      <c r="E153" t="s">
-        <v>14</v>
-      </c>
-      <c r="F153">
-        <v>0.9234</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
-        <v>17</v>
-      </c>
-      <c r="E154" t="s">
-        <v>13</v>
-      </c>
-      <c r="F154">
-        <v>-0.41710000000000003</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
-        <v>17</v>
-      </c>
-      <c r="E155" t="s">
-        <v>14</v>
-      </c>
-      <c r="F155">
-        <v>0.91610000000000003</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
-        <v>21</v>
-      </c>
-      <c r="E156" t="s">
-        <v>13</v>
-      </c>
-      <c r="F156">
-        <v>-0.74150000000000005</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
-        <v>21</v>
-      </c>
-      <c r="E157" t="s">
-        <v>14</v>
-      </c>
-      <c r="F157">
-        <v>0.96550000000000002</v>
-      </c>
-    </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
-        <v>25</v>
-      </c>
-      <c r="E158" t="s">
-        <v>13</v>
-      </c>
-      <c r="F158" s="9">
-        <f>F160</f>
-        <v>-0.58699999999999997</v>
-      </c>
-    </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
-        <v>25</v>
-      </c>
-      <c r="E159" t="s">
-        <v>14</v>
-      </c>
-      <c r="F159" s="9">
-        <f>F161</f>
-        <v>0.82350000000000001</v>
-      </c>
-    </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
-        <v>24</v>
       </c>
       <c r="E160" t="s">
         <v>13</v>
       </c>
       <c r="F160">
+        <v>-0.32340000000000002</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E161" t="s">
+        <v>14</v>
+      </c>
+      <c r="F161">
+        <v>0.97240000000000004</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>16</v>
+      </c>
+      <c r="E162" t="s">
+        <v>13</v>
+      </c>
+      <c r="F162">
+        <v>-0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>16</v>
+      </c>
+      <c r="E163" t="s">
+        <v>14</v>
+      </c>
+      <c r="F163">
+        <v>0.81369999999999998</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>27</v>
+      </c>
+      <c r="E164" t="s">
+        <v>13</v>
+      </c>
+      <c r="F164">
         <v>-0.58699999999999997</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
-        <v>24</v>
-      </c>
-      <c r="E161" t="s">
-        <v>14</v>
-      </c>
-      <c r="F161">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>27</v>
+      </c>
+      <c r="E165" t="s">
+        <v>14</v>
+      </c>
+      <c r="F165">
         <v>0.82350000000000001</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A162" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F162" s="9"/>
-      <c r="H162" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A163" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E163" t="s">
-        <v>14</v>
-      </c>
-      <c r="F163" s="5">
-        <v>1</v>
-      </c>
-      <c r="G163" s="5"/>
-      <c r="H163" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
-        <v>30</v>
-      </c>
-      <c r="E164" t="s">
-        <v>14</v>
-      </c>
-      <c r="F164">
-        <v>1</v>
-      </c>
-      <c r="H164" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
-        <v>31</v>
-      </c>
-      <c r="E165" t="s">
-        <v>14</v>
-      </c>
-      <c r="F165">
-        <v>1</v>
-      </c>
-      <c r="H165" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="E166" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F166">
-        <v>1</v>
-      </c>
-      <c r="H166" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
+        <v>-0.35070000000000001</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E167" t="s">
         <v>14</v>
       </c>
       <c r="F167">
-        <v>1</v>
-      </c>
-      <c r="H167" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
+        <v>0.9234</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E168" t="s">
         <v>13</v>
       </c>
       <c r="F168">
-        <v>-9.2499999999999999E-2</v>
-      </c>
-    </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
+        <v>-0.41710000000000003</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E169" t="s">
         <v>14</v>
       </c>
       <c r="F169">
-        <v>1.2939000000000001</v>
-      </c>
-    </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
+        <v>0.91610000000000003</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E170" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F170">
-        <v>0.94</v>
-      </c>
-      <c r="H170" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
+        <v>-0.74150000000000005</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="E171" t="s">
+        <v>14</v>
+      </c>
+      <c r="F171">
+        <v>0.96550000000000002</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>25</v>
+      </c>
+      <c r="E172" t="s">
         <v>13</v>
       </c>
-      <c r="F171" s="7">
-        <v>-6.83E-2</v>
-      </c>
-      <c r="H171" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
-        <v>36</v>
-      </c>
-      <c r="E172" t="s">
-        <v>14</v>
-      </c>
-      <c r="F172">
-        <v>0.74670000000000003</v>
-      </c>
-    </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F172" s="9">
+        <f>F174</f>
+        <v>-0.58699999999999997</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E173" t="s">
+        <v>14</v>
+      </c>
+      <c r="F173" s="9">
+        <f>F175</f>
+        <v>0.82350000000000001</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>24</v>
+      </c>
+      <c r="E174" t="s">
         <v>13</v>
       </c>
-      <c r="F173" s="9">
-        <f>F171</f>
-        <v>-6.83E-2</v>
-      </c>
-      <c r="H173" s="7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
-        <v>37</v>
-      </c>
-      <c r="E174" t="s">
-        <v>14</v>
-      </c>
-      <c r="F174" s="9">
-        <f>F172</f>
-        <v>0.74670000000000003</v>
-      </c>
-    </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F174">
+        <v>-0.58699999999999997</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="E175" t="s">
         <v>14</v>
       </c>
       <c r="F175">
+        <v>0.82350000000000001</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F176" s="9"/>
+      <c r="H176" s="7"/>
+    </row>
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A177" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E177" t="s">
+        <v>14</v>
+      </c>
+      <c r="F177" s="5">
         <v>1</v>
       </c>
-      <c r="H175" s="5" t="s">
+      <c r="G177" s="5"/>
+      <c r="H177" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A176" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="L176" s="4"/>
-    </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A177" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E177" t="s">
-        <v>13</v>
-      </c>
-      <c r="F177">
-        <v>-8.2500000000000004E-2</v>
-      </c>
-    </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A178" s="10" t="s">
-        <v>40</v>
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>30</v>
       </c>
       <c r="E178" t="s">
         <v>14</v>
       </c>
       <c r="F178">
-        <v>0.72799999999999998</v>
-      </c>
-    </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A179" s="11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A180" s="5" t="s">
-        <v>73</v>
+        <v>1</v>
+      </c>
+      <c r="H178" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>31</v>
+      </c>
+      <c r="E179" t="s">
+        <v>14</v>
+      </c>
+      <c r="F179">
+        <v>1</v>
+      </c>
+      <c r="H179" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>32</v>
       </c>
       <c r="E180" t="s">
         <v>14</v>
@@ -3109,41 +3185,59 @@
         <v>78</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A181" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="H181" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A182" s="11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A183" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A184" s="10" t="s">
-        <v>45</v>
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>33</v>
+      </c>
+      <c r="E181" t="s">
+        <v>14</v>
+      </c>
+      <c r="F181">
+        <v>1</v>
+      </c>
+      <c r="H181" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>34</v>
+      </c>
+      <c r="E182" t="s">
+        <v>13</v>
+      </c>
+      <c r="F182">
+        <v>-9.2499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>34</v>
+      </c>
+      <c r="E183" t="s">
+        <v>14</v>
+      </c>
+      <c r="F183">
+        <v>1.2939000000000001</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>35</v>
       </c>
       <c r="E184" t="s">
         <v>14</v>
       </c>
       <c r="F184">
-        <v>1</v>
+        <v>0.94</v>
       </c>
       <c r="H184" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A185" s="10" t="s">
-        <v>46</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>36</v>
       </c>
       <c r="E185" t="s">
         <v>14</v>
@@ -3155,9 +3249,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E186" t="s">
         <v>14</v>
@@ -3169,9 +3263,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E187" t="s">
         <v>14</v>
@@ -3183,65 +3277,42 @@
         <v>78</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A188" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E188" t="s">
-        <v>14</v>
-      </c>
-      <c r="F188">
-        <v>1</v>
-      </c>
-      <c r="H188" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A189" s="5" t="s">
-        <v>50</v>
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A188" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="L188" s="4"/>
+    </row>
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A189" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="E189" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F189">
-        <v>1</v>
-      </c>
-      <c r="H189" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A190" s="5" t="s">
-        <v>51</v>
+        <v>-8.2500000000000004E-2</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A190" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="E190" t="s">
         <v>14</v>
       </c>
       <c r="F190">
-        <v>1</v>
-      </c>
-      <c r="H190" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A191" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E191" t="s">
-        <v>14</v>
-      </c>
-      <c r="F191">
-        <v>1</v>
-      </c>
-      <c r="H191" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.72799999999999998</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A191" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" s="5" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E192" t="s">
         <v>14</v>
@@ -3254,64 +3325,42 @@
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A193" s="5" t="s">
-        <v>54</v>
+      <c r="A193" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="E193" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F193">
-        <v>1</v>
-      </c>
-      <c r="H193" s="5" t="s">
-        <v>78</v>
-      </c>
+        <v>-3.2399999999999998E-2</v>
+      </c>
+      <c r="H193" s="7"/>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A194" s="5" t="s">
-        <v>55</v>
+      <c r="A194" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="E194" t="s">
         <v>14</v>
       </c>
       <c r="F194">
-        <v>1</v>
-      </c>
-      <c r="H194" s="5" t="s">
-        <v>78</v>
-      </c>
+        <v>0.82120000000000004</v>
+      </c>
+      <c r="H194" s="7"/>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A195" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E195" t="s">
-        <v>14</v>
-      </c>
-      <c r="F195">
-        <v>1</v>
-      </c>
-      <c r="H195" s="5" t="s">
-        <v>78</v>
+      <c r="A195" s="11" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A196" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E196" t="s">
-        <v>14</v>
-      </c>
-      <c r="F196">
-        <v>1</v>
-      </c>
-      <c r="H196" s="5" t="s">
-        <v>78</v>
+      <c r="A196" s="11" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A197" s="5" t="s">
-        <v>58</v>
+      <c r="A197" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="E197" t="s">
         <v>14</v>
@@ -3324,8 +3373,8 @@
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A198" s="5" t="s">
-        <v>59</v>
+      <c r="A198" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="E198" t="s">
         <v>14</v>
@@ -3338,8 +3387,8 @@
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A199" s="5" t="s">
-        <v>60</v>
+      <c r="A199" t="s">
+        <v>47</v>
       </c>
       <c r="E199" t="s">
         <v>14</v>
@@ -3352,8 +3401,8 @@
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A200" s="5" t="s">
-        <v>61</v>
+      <c r="A200" t="s">
+        <v>48</v>
       </c>
       <c r="E200" t="s">
         <v>14</v>
@@ -3367,7 +3416,7 @@
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="5" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="E201" t="s">
         <v>14</v>
@@ -3381,7 +3430,7 @@
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="5" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="E202" t="s">
         <v>14</v>
@@ -3395,7 +3444,7 @@
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="5" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="E203" t="s">
         <v>14</v>
@@ -3409,7 +3458,7 @@
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="5" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="E204" t="s">
         <v>14</v>
@@ -3423,7 +3472,7 @@
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="E205" t="s">
         <v>14</v>
@@ -3437,7 +3486,7 @@
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="5" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E206" t="s">
         <v>14</v>
@@ -3451,7 +3500,7 @@
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="5" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="E207" t="s">
         <v>14</v>
@@ -3465,7 +3514,7 @@
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="5" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="E208" t="s">
         <v>14</v>
@@ -3479,7 +3528,7 @@
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="5" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E209" t="s">
         <v>14</v>
@@ -3493,7 +3542,7 @@
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="5" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="E210" t="s">
         <v>14</v>
@@ -3507,7 +3556,7 @@
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E211" t="s">
         <v>14</v>
@@ -3516,6 +3565,188 @@
         <v>1</v>
       </c>
       <c r="H211" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A212" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E212" t="s">
+        <v>14</v>
+      </c>
+      <c r="F212">
+        <v>1</v>
+      </c>
+      <c r="H212" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A213" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E213" t="s">
+        <v>14</v>
+      </c>
+      <c r="F213">
+        <v>1</v>
+      </c>
+      <c r="H213" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A214" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E214" t="s">
+        <v>14</v>
+      </c>
+      <c r="F214">
+        <v>1</v>
+      </c>
+      <c r="H214" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A215" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E215" t="s">
+        <v>14</v>
+      </c>
+      <c r="F215">
+        <v>1</v>
+      </c>
+      <c r="H215" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A216" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E216" t="s">
+        <v>14</v>
+      </c>
+      <c r="F216">
+        <v>1</v>
+      </c>
+      <c r="H216" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A217" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E217" t="s">
+        <v>14</v>
+      </c>
+      <c r="F217">
+        <v>1</v>
+      </c>
+      <c r="H217" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A218" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E218" t="s">
+        <v>14</v>
+      </c>
+      <c r="F218">
+        <v>1</v>
+      </c>
+      <c r="H218" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A219" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E219" t="s">
+        <v>14</v>
+      </c>
+      <c r="F219">
+        <v>1</v>
+      </c>
+      <c r="H219" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A220" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E220" t="s">
+        <v>14</v>
+      </c>
+      <c r="F220">
+        <v>1</v>
+      </c>
+      <c r="H220" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A221" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E221" t="s">
+        <v>14</v>
+      </c>
+      <c r="F221">
+        <v>1</v>
+      </c>
+      <c r="H221" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A222" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E222" t="s">
+        <v>14</v>
+      </c>
+      <c r="F222">
+        <v>1</v>
+      </c>
+      <c r="H222" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A223" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E223" t="s">
+        <v>14</v>
+      </c>
+      <c r="F223">
+        <v>1</v>
+      </c>
+      <c r="H223" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A224" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E224" t="s">
+        <v>14</v>
+      </c>
+      <c r="F224">
+        <v>1</v>
+      </c>
+      <c r="H224" s="5" t="s">
         <v>78</v>
       </c>
     </row>
@@ -3535,7 +3766,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3543,7 +3774,7 @@
         <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3551,7 +3782,7 @@
         <v>112</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3559,7 +3790,7 @@
         <v>311</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3567,7 +3798,7 @@
         <v>312</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3575,7 +3806,7 @@
         <v>321</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3583,7 +3814,7 @@
         <v>322</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3591,7 +3822,7 @@
         <v>411</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3599,7 +3830,7 @@
         <v>421</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3607,7 +3838,7 @@
         <v>422</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3615,7 +3846,7 @@
         <v>431</v>
       </c>
       <c r="B11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3623,7 +3854,7 @@
         <v>511</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3631,7 +3862,7 @@
         <v>512</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3639,7 +3870,7 @@
         <v>513</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3647,7 +3878,7 @@
         <v>514</v>
       </c>
       <c r="B15" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3655,7 +3886,7 @@
         <v>515</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3663,7 +3894,7 @@
         <v>521</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3671,7 +3902,7 @@
         <v>611</v>
       </c>
       <c r="B18" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3679,7 +3910,7 @@
         <v>612</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3687,7 +3918,7 @@
         <v>621</v>
       </c>
       <c r="B20" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3695,7 +3926,7 @@
         <v>622</v>
       </c>
       <c r="B21" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3703,7 +3934,7 @@
         <v>711</v>
       </c>
       <c r="B22" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3711,7 +3942,7 @@
         <v>731</v>
       </c>
       <c r="B23" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3719,7 +3950,7 @@
         <v>811</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3727,7 +3958,7 @@
         <v>812</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3735,7 +3966,7 @@
         <v>813</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3743,7 +3974,7 @@
         <v>814</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3751,7 +3982,7 @@
         <v>821</v>
       </c>
       <c r="B28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -3759,7 +3990,7 @@
         <v>831</v>
       </c>
       <c r="B29" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3767,7 +3998,7 @@
         <v>911</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3775,7 +4006,7 @@
         <v>912</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -3783,7 +4014,7 @@
         <v>913</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3791,7 +4022,7 @@
         <v>1011</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -3799,7 +4030,7 @@
         <v>1111</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -3807,7 +4038,7 @@
         <v>1112</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -3815,7 +4046,7 @@
         <v>1121</v>
       </c>
       <c r="B36" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3823,7 +4054,7 @@
         <v>1122</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -3831,7 +4062,7 @@
         <v>1123</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -3839,7 +4070,7 @@
         <v>1124</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -3847,7 +4078,7 @@
         <v>1131</v>
       </c>
       <c r="B40" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -3855,7 +4086,7 @@
         <v>1211</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3863,7 +4094,7 @@
         <v>1212</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3871,7 +4102,7 @@
         <v>1213</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -3879,7 +4110,7 @@
         <v>1214</v>
       </c>
       <c r="B44" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -3887,7 +4118,7 @@
         <v>1215</v>
       </c>
       <c r="B45" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -3895,7 +4126,7 @@
         <v>1216</v>
       </c>
       <c r="B46" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -3903,7 +4134,7 @@
         <v>1221</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -3911,7 +4142,7 @@
         <v>1222</v>
       </c>
       <c r="B48" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -3919,7 +4150,7 @@
         <v>1311</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -3927,7 +4158,7 @@
         <v>1321</v>
       </c>
       <c r="B50" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -3935,7 +4166,7 @@
         <v>1322</v>
       </c>
       <c r="B51" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -3943,7 +4174,7 @@
         <v>1331</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -3951,7 +4182,7 @@
         <v>1411</v>
       </c>
       <c r="B53" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -3959,7 +4190,7 @@
         <v>1412</v>
       </c>
       <c r="B54" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -3967,7 +4198,7 @@
         <v>1421</v>
       </c>
       <c r="B55" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -3975,7 +4206,7 @@
         <v>1511</v>
       </c>
       <c r="B56" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -3983,7 +4214,7 @@
         <v>1512</v>
       </c>
       <c r="B57" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -3991,7 +4222,7 @@
         <v>1521</v>
       </c>
       <c r="B58" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -3999,7 +4230,7 @@
         <v>1522</v>
       </c>
       <c r="B59" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -4007,7 +4238,7 @@
         <v>1611</v>
       </c>
       <c r="B60" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -4015,7 +4246,7 @@
         <v>1612</v>
       </c>
       <c r="B61" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -4023,7 +4254,7 @@
         <v>1613</v>
       </c>
       <c r="B62" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -4031,7 +4262,7 @@
         <v>1614</v>
       </c>
       <c r="B63" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -4039,7 +4270,7 @@
         <v>1615</v>
       </c>
       <c r="B64" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -4047,7 +4278,7 @@
         <v>1616</v>
       </c>
       <c r="B65" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -4055,7 +4286,7 @@
         <v>1617</v>
       </c>
       <c r="B66" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -4063,7 +4294,7 @@
         <v>1621</v>
       </c>
       <c r="B67" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -4071,7 +4302,7 @@
         <v>1622</v>
       </c>
       <c r="B68" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -4079,7 +4310,7 @@
         <v>1623</v>
       </c>
       <c r="B69" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -4087,7 +4318,7 @@
         <v>1711</v>
       </c>
       <c r="B70" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -4095,7 +4326,7 @@
         <v>1712</v>
       </c>
       <c r="B71" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -4103,7 +4334,7 @@
         <v>1713</v>
       </c>
       <c r="B72" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -4111,7 +4342,7 @@
         <v>1721</v>
       </c>
       <c r="B73" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -4119,7 +4350,7 @@
         <v>1722</v>
       </c>
       <c r="B74" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -4127,7 +4358,7 @@
         <v>1723</v>
       </c>
       <c r="B75" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -4135,7 +4366,7 @@
         <v>1724</v>
       </c>
       <c r="B76" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -4143,7 +4374,7 @@
         <v>1811</v>
       </c>
       <c r="B77" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -4151,7 +4382,7 @@
         <v>1812</v>
       </c>
       <c r="B78" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -4159,7 +4390,7 @@
         <v>1813</v>
       </c>
       <c r="B79" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -4167,7 +4398,7 @@
         <v>1821</v>
       </c>
       <c r="B80" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -4175,7 +4406,7 @@
         <v>1911</v>
       </c>
       <c r="B81" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -4183,7 +4414,7 @@
         <v>1912</v>
       </c>
       <c r="B82" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -4191,7 +4422,7 @@
         <v>1921</v>
       </c>
       <c r="B83" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -4199,7 +4430,7 @@
         <v>1922</v>
       </c>
       <c r="B84" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -4207,7 +4438,7 @@
         <v>2011</v>
       </c>
       <c r="B85" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -4215,7 +4446,7 @@
         <v>2012</v>
       </c>
       <c r="B86" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -4223,7 +4454,7 @@
         <v>2019</v>
       </c>
       <c r="B87" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -4231,7 +4462,7 @@
         <v>2111</v>
       </c>
       <c r="B88" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -4239,7 +4470,7 @@
         <v>2121</v>
       </c>
       <c r="B89" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -4247,7 +4478,7 @@
         <v>2122</v>
       </c>
       <c r="B90" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -4255,7 +4486,7 @@
         <v>2211</v>
       </c>
       <c r="B91" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -4263,7 +4494,7 @@
         <v>2212</v>
       </c>
       <c r="B92" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -4271,7 +4502,7 @@
         <v>2221</v>
       </c>
       <c r="B93" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -4279,7 +4510,7 @@
         <v>2311</v>
       </c>
       <c r="B94" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -4287,7 +4518,7 @@
         <v>2312</v>
       </c>
       <c r="B95" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -4295,7 +4526,7 @@
         <v>2319</v>
       </c>
       <c r="B96" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -4303,7 +4534,7 @@
         <v>2331</v>
       </c>
       <c r="B97" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -4311,7 +4542,7 @@
         <v>2411</v>
       </c>
       <c r="B98" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -4319,7 +4550,7 @@
         <v>2412</v>
       </c>
       <c r="B99" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -4327,7 +4558,7 @@
         <v>2413</v>
       </c>
       <c r="B100" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -4335,7 +4566,7 @@
         <v>2414</v>
       </c>
       <c r="B101" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -4343,7 +4574,7 @@
         <v>2415</v>
       </c>
       <c r="B102" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -4351,7 +4582,7 @@
         <v>2419</v>
       </c>
       <c r="B103" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -4359,7 +4590,7 @@
         <v>2511</v>
       </c>
       <c r="B104" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -4367,7 +4598,7 @@
         <v>2512</v>
       </c>
       <c r="B105" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -4375,7 +4606,7 @@
         <v>2519</v>
       </c>
       <c r="B106" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -4383,7 +4614,7 @@
         <v>2521</v>
       </c>
       <c r="B107" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added parameters for some crops
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FertiliserMgmt.xlsx
+++ b/data/prod_parameters/FertiliserMgmt.xlsx
@@ -10,7 +10,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="relations" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="115">
   <si>
     <t>f_crop</t>
   </si>
@@ -380,6 +380,15 @@
   </si>
   <si>
     <t>Potatis</t>
+  </si>
+  <si>
+    <t>Assume same as apples</t>
+  </si>
+  <si>
+    <t>Assume same as carrots</t>
+  </si>
+  <si>
+    <t>Assume same as lettuce</t>
   </si>
 </sst>
 </file>
@@ -768,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L224"/>
+  <dimension ref="A1:L226"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
@@ -2611,25 +2620,30 @@
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" s="7" t="s">
+      <c r="A126" s="5" t="s">
         <v>49</v>
+      </c>
+      <c r="E126" t="s">
+        <v>11</v>
+      </c>
+      <c r="F126" s="9">
+        <f>F124</f>
+        <v>1.3846000000000001</v>
+      </c>
+      <c r="H126" s="7" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E127" t="s">
-        <v>11</v>
-      </c>
-      <c r="F127">
-        <v>3.3332999999999999</v>
-      </c>
-      <c r="H127" t="s">
-        <v>87</v>
-      </c>
-      <c r="I127" t="s">
-        <v>86</v>
+        <v>12</v>
+      </c>
+      <c r="F127" s="9">
+        <f>F125</f>
+        <v>11.538</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -2637,27 +2651,27 @@
         <v>50</v>
       </c>
       <c r="E128" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F128">
-        <v>33.332999999999998</v>
+        <v>3.3332999999999999</v>
+      </c>
+      <c r="H128" t="s">
+        <v>87</v>
+      </c>
+      <c r="I128" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E129" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F129">
-        <v>3</v>
-      </c>
-      <c r="H129" t="s">
-        <v>88</v>
-      </c>
-      <c r="I129" t="s">
-        <v>86</v>
+        <v>33.332999999999998</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -2665,38 +2679,44 @@
         <v>51</v>
       </c>
       <c r="E130" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F130">
-        <v>90</v>
+        <v>3</v>
+      </c>
+      <c r="H130" t="s">
+        <v>88</v>
+      </c>
+      <c r="I130" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E131" s="5" t="s">
-        <v>10</v>
+        <v>51</v>
+      </c>
+      <c r="E131" t="s">
+        <v>12</v>
       </c>
       <c r="F131">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="H131" t="s">
-        <v>89</v>
-      </c>
-      <c r="I131" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E132" t="s">
-        <v>11</v>
+      <c r="E132" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="F132">
-        <v>1.2583</v>
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H132" t="s">
+        <v>89</v>
+      </c>
+      <c r="I132" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -2704,94 +2724,108 @@
         <v>52</v>
       </c>
       <c r="E133" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F133">
-        <v>0</v>
+        <v>1.2583</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F134" s="9">
-        <f>F131</f>
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="H134" s="9" t="str">
-        <f>H131</f>
-        <v xml:space="preserve">yield in fresh weight 5% DM </v>
-      </c>
-      <c r="I134" s="9" t="str">
-        <f>I131</f>
-        <v>Yara (2018)</v>
+        <v>52</v>
+      </c>
+      <c r="E134" t="s">
+        <v>12</v>
+      </c>
+      <c r="F134">
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E135" t="s">
-        <v>11</v>
+      <c r="E135" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="F135" s="9">
         <f>F132</f>
-        <v>1.2583</v>
-      </c>
-      <c r="G135" s="9"/>
-      <c r="H135" s="9"/>
-      <c r="I135" s="9"/>
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H135" s="9" t="str">
+        <f>H132</f>
+        <v xml:space="preserve">yield in fresh weight 5% DM </v>
+      </c>
+      <c r="I135" s="9" t="str">
+        <f>I132</f>
+        <v>Yara (2018)</v>
+      </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
         <v>53</v>
       </c>
       <c r="E136" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F136" s="9">
         <f>F133</f>
-        <v>0</v>
+        <v>1.2583</v>
       </c>
       <c r="G136" s="9"/>
       <c r="H136" s="9"/>
       <c r="I136" s="9"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A137" s="7" t="s">
+      <c r="A137" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E137" t="s">
+        <v>12</v>
+      </c>
+      <c r="F137" s="9">
+        <f>F134</f>
+        <v>0</v>
+      </c>
+      <c r="G137" s="9"/>
+      <c r="H137" s="9"/>
+      <c r="I137" s="9"/>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A138" s="5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138" s="7" t="s">
-        <v>55</v>
+      <c r="E138" t="s">
+        <v>11</v>
+      </c>
+      <c r="F138" s="9">
+        <f>F128</f>
+        <v>3.3332999999999999</v>
+      </c>
+      <c r="H138" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E139" t="s">
         <v>12</v>
       </c>
-      <c r="F139">
-        <v>65</v>
-      </c>
-      <c r="H139" t="s">
-        <v>82</v>
+      <c r="F139" s="9">
+        <f>F129</f>
+        <v>33.332999999999998</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E141" t="s">
         <v>12</v>
@@ -2800,380 +2834,381 @@
         <v>65</v>
       </c>
       <c r="H141" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A142" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E142" t="s">
-        <v>12</v>
-      </c>
-      <c r="F142">
-        <v>100</v>
-      </c>
-      <c r="H142" t="s">
-        <v>84</v>
+      <c r="A142" s="7" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E143" t="s">
+        <v>12</v>
+      </c>
+      <c r="F143">
+        <v>65</v>
+      </c>
+      <c r="H143" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E144" t="s">
+        <v>12</v>
+      </c>
+      <c r="F144">
+        <v>100</v>
+      </c>
+      <c r="H144" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A145" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E143" t="s">
-        <v>12</v>
-      </c>
-      <c r="F143">
+      <c r="E145" t="s">
+        <v>12</v>
+      </c>
+      <c r="F145">
         <v>110</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A144" s="7" t="s">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A146" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A145" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A146" s="7" t="s">
-        <v>63</v>
+      <c r="E146" t="s">
+        <v>12</v>
+      </c>
+      <c r="F146" s="9">
+        <f>F144</f>
+        <v>100</v>
+      </c>
+      <c r="H146" s="7" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A152" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E152" t="s">
-        <v>12</v>
-      </c>
-      <c r="F152">
-        <v>0</v>
-      </c>
-      <c r="H152" t="s">
-        <v>74</v>
+      <c r="A152" s="7" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A154" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E154" t="s">
+        <v>12</v>
+      </c>
+      <c r="F154">
+        <v>0</v>
+      </c>
+      <c r="H154" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A155" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A154" s="7" t="s">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A156" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A155" s="5" t="s">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A157" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E155" t="s">
-        <v>12</v>
-      </c>
-      <c r="F155">
+      <c r="E157" t="s">
+        <v>12</v>
+      </c>
+      <c r="F157">
         <v>0</v>
       </c>
-      <c r="H155" t="s">
+      <c r="H157" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A157" s="2" t="s">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B157" s="2"/>
-      <c r="C157" s="2"/>
-      <c r="D157" s="2"/>
-      <c r="E157" s="2"/>
-      <c r="F157" s="2"/>
-      <c r="G157" s="2"/>
-      <c r="H157" s="3"/>
-      <c r="I157" s="3"/>
-    </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E158" s="6" t="s">
+      <c r="B159" s="2"/>
+      <c r="C159" s="2"/>
+      <c r="D159" s="2"/>
+      <c r="E159" s="2"/>
+      <c r="F159" s="2"/>
+      <c r="G159" s="2"/>
+      <c r="H159" s="3"/>
+      <c r="I159" s="3"/>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E160" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F158" s="6">
+      <c r="F160" s="6">
         <v>0</v>
       </c>
-      <c r="G158" s="6"/>
-      <c r="H158" s="6" t="s">
+      <c r="G160" s="6"/>
+      <c r="H160" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E159" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F159" s="6">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E161" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F161" s="6">
         <v>1</v>
       </c>
-      <c r="G159" s="6"/>
-      <c r="H159" s="6" t="s">
+      <c r="G161" s="6"/>
+      <c r="H161" s="6" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
-        <v>7</v>
-      </c>
-      <c r="E160" t="s">
-        <v>13</v>
-      </c>
-      <c r="F160">
-        <v>-0.32340000000000002</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
-        <v>7</v>
-      </c>
-      <c r="E161" t="s">
-        <v>14</v>
-      </c>
-      <c r="F161">
-        <v>0.97240000000000004</v>
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E162" t="s">
         <v>13</v>
       </c>
       <c r="F162">
-        <v>-0.32500000000000001</v>
+        <v>-0.32340000000000002</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E163" t="s">
         <v>14</v>
       </c>
       <c r="F163">
-        <v>0.81369999999999998</v>
+        <v>0.97240000000000004</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E164" t="s">
         <v>13</v>
       </c>
       <c r="F164">
-        <v>-0.58699999999999997</v>
+        <v>-0.32500000000000001</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E165" t="s">
         <v>14</v>
       </c>
       <c r="F165">
-        <v>0.82350000000000001</v>
+        <v>0.81369999999999998</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E166" t="s">
         <v>13</v>
       </c>
       <c r="F166">
-        <v>-0.35070000000000001</v>
+        <v>-0.58699999999999997</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E167" t="s">
         <v>14</v>
       </c>
       <c r="F167">
-        <v>0.9234</v>
+        <v>0.82350000000000001</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E168" t="s">
         <v>13</v>
       </c>
       <c r="F168">
-        <v>-0.41710000000000003</v>
+        <v>-0.35070000000000001</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E169" t="s">
         <v>14</v>
       </c>
       <c r="F169">
-        <v>0.91610000000000003</v>
+        <v>0.9234</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E170" t="s">
         <v>13</v>
       </c>
       <c r="F170">
-        <v>-0.74150000000000005</v>
+        <v>-0.41710000000000003</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E171" t="s">
         <v>14</v>
       </c>
       <c r="F171">
-        <v>0.96550000000000002</v>
+        <v>0.91610000000000003</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E172" t="s">
         <v>13</v>
       </c>
-      <c r="F172" s="9">
-        <f>F174</f>
-        <v>-0.58699999999999997</v>
+      <c r="F172">
+        <v>-0.74150000000000005</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E173" t="s">
         <v>14</v>
       </c>
-      <c r="F173" s="9">
-        <f>F175</f>
-        <v>0.82350000000000001</v>
+      <c r="F173">
+        <v>0.96550000000000002</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E174" t="s">
         <v>13</v>
       </c>
-      <c r="F174">
+      <c r="F174" s="9">
+        <f>F176</f>
         <v>-0.58699999999999997</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>25</v>
+      </c>
+      <c r="E175" t="s">
+        <v>14</v>
+      </c>
+      <c r="F175" s="9">
+        <f>F177</f>
+        <v>0.82350000000000001</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
         <v>24</v>
       </c>
-      <c r="E175" t="s">
-        <v>14</v>
-      </c>
-      <c r="F175">
+      <c r="E176" t="s">
+        <v>13</v>
+      </c>
+      <c r="F176">
+        <v>-0.58699999999999997</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>24</v>
+      </c>
+      <c r="E177" t="s">
+        <v>14</v>
+      </c>
+      <c r="F177">
         <v>0.82350000000000001</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A176" s="7" t="s">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A178" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F176" s="9"/>
-      <c r="H176" s="7"/>
-    </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A177" s="5" t="s">
+      <c r="F178" s="9"/>
+      <c r="H178" s="7"/>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A179" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E177" t="s">
-        <v>14</v>
-      </c>
-      <c r="F177" s="5">
+      <c r="E179" t="s">
+        <v>14</v>
+      </c>
+      <c r="F179" s="5">
         <v>1</v>
       </c>
-      <c r="G177" s="5"/>
-      <c r="H177" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
-        <v>30</v>
-      </c>
-      <c r="E178" t="s">
-        <v>14</v>
-      </c>
-      <c r="F178">
-        <v>1</v>
-      </c>
-      <c r="H178" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
-        <v>31</v>
-      </c>
-      <c r="E179" t="s">
-        <v>14</v>
-      </c>
-      <c r="F179">
-        <v>1</v>
-      </c>
+      <c r="G179" s="5"/>
       <c r="H179" s="5" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E180" t="s">
         <v>14</v>
@@ -3187,7 +3222,7 @@
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E181" t="s">
         <v>14</v>
@@ -3201,71 +3236,71 @@
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E182" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F182">
-        <v>-9.2499999999999999E-2</v>
+        <v>1</v>
+      </c>
+      <c r="H182" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E183" t="s">
         <v>14</v>
       </c>
       <c r="F183">
-        <v>1.2939000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="H183" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E184" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F184">
-        <v>0.94</v>
-      </c>
-      <c r="H184" s="5" t="s">
-        <v>79</v>
+        <v>-9.2499999999999999E-2</v>
       </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E185" t="s">
         <v>14</v>
       </c>
       <c r="F185">
-        <v>1</v>
-      </c>
-      <c r="H185" s="5" t="s">
-        <v>78</v>
+        <v>1.2939000000000001</v>
       </c>
     </row>
     <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E186" t="s">
         <v>14</v>
       </c>
       <c r="F186">
-        <v>1</v>
+        <v>0.94</v>
       </c>
       <c r="H186" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E187" t="s">
         <v>14</v>
@@ -3278,117 +3313,117 @@
       </c>
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A188" s="7" t="s">
+      <c r="A188" t="s">
+        <v>37</v>
+      </c>
+      <c r="E188" t="s">
+        <v>14</v>
+      </c>
+      <c r="F188">
+        <v>1</v>
+      </c>
+      <c r="H188" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>38</v>
+      </c>
+      <c r="E189" t="s">
+        <v>14</v>
+      </c>
+      <c r="F189">
+        <v>1</v>
+      </c>
+      <c r="H189" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A190" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="L188" s="4"/>
-    </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A189" s="10" t="s">
+      <c r="L190" s="4"/>
+    </row>
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A191" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E189" t="s">
+      <c r="E191" t="s">
         <v>13</v>
       </c>
-      <c r="F189">
+      <c r="F191">
         <v>-8.2500000000000004E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A190" s="10" t="s">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A192" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E190" t="s">
-        <v>14</v>
-      </c>
-      <c r="F190">
+      <c r="E192" t="s">
+        <v>14</v>
+      </c>
+      <c r="F192">
         <v>0.72799999999999998</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A191" s="11" t="s">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A193" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A192" s="5" t="s">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A194" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E192" t="s">
-        <v>14</v>
-      </c>
-      <c r="F192">
+      <c r="E194" t="s">
+        <v>14</v>
+      </c>
+      <c r="F194">
         <v>1</v>
       </c>
-      <c r="H192" s="5" t="s">
+      <c r="H194" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A193" s="10" t="s">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A195" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E193" t="s">
+      <c r="E195" t="s">
         <v>13</v>
       </c>
-      <c r="F193">
+      <c r="F195">
         <v>-3.2399999999999998E-2</v>
       </c>
-      <c r="H193" s="7"/>
-    </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A194" s="10" t="s">
+      <c r="H195" s="7"/>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A196" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E194" t="s">
-        <v>14</v>
-      </c>
-      <c r="F194">
+      <c r="E196" t="s">
+        <v>14</v>
+      </c>
+      <c r="F196">
         <v>0.82120000000000004</v>
       </c>
-      <c r="H194" s="7"/>
-    </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A195" s="11" t="s">
+      <c r="H196" s="7"/>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A197" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A196" s="11" t="s">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A198" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A197" s="10" t="s">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A199" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="E197" t="s">
-        <v>14</v>
-      </c>
-      <c r="F197">
-        <v>1</v>
-      </c>
-      <c r="H197" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A198" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E198" t="s">
-        <v>14</v>
-      </c>
-      <c r="F198">
-        <v>1</v>
-      </c>
-      <c r="H198" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A199" t="s">
-        <v>47</v>
       </c>
       <c r="E199" t="s">
         <v>14</v>
@@ -3401,8 +3436,8 @@
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A200" t="s">
-        <v>48</v>
+      <c r="A200" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="E200" t="s">
         <v>14</v>
@@ -3415,8 +3450,8 @@
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A201" s="5" t="s">
-        <v>49</v>
+      <c r="A201" t="s">
+        <v>47</v>
       </c>
       <c r="E201" t="s">
         <v>14</v>
@@ -3429,8 +3464,8 @@
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A202" s="5" t="s">
-        <v>50</v>
+      <c r="A202" t="s">
+        <v>48</v>
       </c>
       <c r="E202" t="s">
         <v>14</v>
@@ -3444,7 +3479,7 @@
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E203" t="s">
         <v>14</v>
@@ -3458,7 +3493,7 @@
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E204" t="s">
         <v>14</v>
@@ -3472,7 +3507,7 @@
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E205" t="s">
         <v>14</v>
@@ -3486,7 +3521,7 @@
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E206" t="s">
         <v>14</v>
@@ -3500,7 +3535,7 @@
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E207" t="s">
         <v>14</v>
@@ -3514,7 +3549,7 @@
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E208" t="s">
         <v>14</v>
@@ -3528,7 +3563,7 @@
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E209" t="s">
         <v>14</v>
@@ -3542,7 +3577,7 @@
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E210" t="s">
         <v>14</v>
@@ -3556,7 +3591,7 @@
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E211" t="s">
         <v>14</v>
@@ -3570,7 +3605,7 @@
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E212" t="s">
         <v>14</v>
@@ -3584,7 +3619,7 @@
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E213" t="s">
         <v>14</v>
@@ -3598,7 +3633,7 @@
     </row>
     <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E214" t="s">
         <v>14</v>
@@ -3612,7 +3647,7 @@
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E215" t="s">
         <v>14</v>
@@ -3626,7 +3661,7 @@
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E216" t="s">
         <v>14</v>
@@ -3640,7 +3675,7 @@
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E217" t="s">
         <v>14</v>
@@ -3654,7 +3689,7 @@
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E218" t="s">
         <v>14</v>
@@ -3668,7 +3703,7 @@
     </row>
     <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E219" t="s">
         <v>14</v>
@@ -3682,7 +3717,7 @@
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E220" t="s">
         <v>14</v>
@@ -3696,7 +3731,7 @@
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E221" t="s">
         <v>14</v>
@@ -3710,7 +3745,7 @@
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E222" t="s">
         <v>14</v>
@@ -3724,7 +3759,7 @@
     </row>
     <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E223" t="s">
         <v>14</v>
@@ -3738,7 +3773,7 @@
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E224" t="s">
         <v>14</v>
@@ -3747,6 +3782,34 @@
         <v>1</v>
       </c>
       <c r="H224" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A225" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E225" t="s">
+        <v>14</v>
+      </c>
+      <c r="F225">
+        <v>1</v>
+      </c>
+      <c r="H225" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A226" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E226" t="s">
+        <v>14</v>
+      </c>
+      <c r="F226">
+        <v>1</v>
+      </c>
+      <c r="H226" s="5" t="s">
         <v>78</v>
       </c>
     </row>

</xml_diff>